<commit_message>
Fix & Polish: Natürliches Schüler-Design ohne Textüberlauf in Excel und PowerPoint; Nutzwertanalysen mathematisch korrigiert (Gewinner matchen Score); Strukturplan und Netzplan mit vollem Text lesbar
</commit_message>
<xml_diff>
--- a/docs/03_Marktrecherche/Nutzwertanalyse_Monitore.xlsx
+++ b/docs/03_Marktrecherche/Nutzwertanalyse_Monitore.xlsx
@@ -7,7 +7,7 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="NWA Monitore" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Nutzwertanalyse Monitore" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -17,7 +17,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="5">
+  <fonts count="10">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -26,16 +26,52 @@
       <scheme val="minor"/>
     </font>
     <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="001F497D"/>
+      <sz val="14"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <i val="1"/>
+      <color rgb="00595959"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
       <b val="1"/>
       <color rgb="00FFFFFF"/>
-    </font>
-    <font/>
-    <font>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
       <b val="1"/>
-    </font>
-    <font>
+      <sz val="11"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
       <b val="1"/>
-      <color rgb="00006100"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="00276A3C"/>
+      <sz val="12"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="00276A3C"/>
+      <sz val="10.5"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <sz val="9.5"/>
     </font>
   </fonts>
   <fills count="4">
@@ -47,18 +83,16 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00E26B0A"/>
-        <bgColor rgb="00E26B0A"/>
+        <fgColor rgb="001F497D"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00C6EFCE"/>
-        <bgColor rgb="00C6EFCE"/>
+        <fgColor rgb="00E2EFDA"/>
       </patternFill>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="3">
     <border>
       <left/>
       <right/>
@@ -68,15 +102,23 @@
     </border>
     <border>
       <left style="thin">
-        <color rgb="00000000"/>
+        <color rgb="00D9D9D9"/>
       </left>
       <right style="thin">
-        <color rgb="00000000"/>
+        <color rgb="00D9D9D9"/>
       </right>
       <top style="thin">
+        <color rgb="00D9D9D9"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00D9D9D9"/>
+      </bottom>
+    </border>
+    <border>
+      <top style="medium">
         <color rgb="00000000"/>
       </top>
-      <bottom style="thin">
+      <bottom style="double">
         <color rgb="00000000"/>
       </bottom>
     </border>
@@ -84,27 +126,41 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="18">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="9" fontId="4" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="9" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center"/>
+    <xf numFmtId="2" fontId="4" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="9" fontId="6" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="9" fontId="3" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="2" fontId="7" fillId="3" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center"/>
+    <xf numFmtId="2" fontId="5" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -470,275 +526,332 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H10"/>
+  <dimension ref="A1:H19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="78" customWidth="1" min="1" max="1"/>
-    <col width="13" customWidth="1" min="2" max="2"/>
-    <col width="20" customWidth="1" min="3" max="3"/>
-    <col width="20" customWidth="1" min="4" max="4"/>
-    <col width="23" customWidth="1" min="5" max="5"/>
-    <col width="23" customWidth="1" min="6" max="6"/>
-    <col width="20" customWidth="1" min="7" max="7"/>
-    <col width="20" customWidth="1" min="8" max="8"/>
+    <col width="34" customWidth="1" min="1" max="1"/>
+    <col width="12" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
+    <col width="14" customWidth="1" min="4" max="4"/>
+    <col width="14" customWidth="1" min="5" max="5"/>
+    <col width="14" customWidth="1" min="6" max="6"/>
+    <col width="14" customWidth="1" min="7" max="7"/>
+    <col width="14" customWidth="1" min="8" max="8"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Kriterium</t>
-        </is>
-      </c>
-      <c r="B1" s="1" t="inlineStr">
-        <is>
-          <t>Gewichtung</t>
-        </is>
-      </c>
-      <c r="C1" s="1" t="inlineStr">
-        <is>
-          <t>Dell U2724D (Note)</t>
-        </is>
-      </c>
-      <c r="D1" s="1" t="inlineStr">
-        <is>
-          <t>Dell U2724D (Wert)</t>
-        </is>
-      </c>
-      <c r="E1" s="1" t="inlineStr">
-        <is>
-          <t>Lenovo P27h-30 (Note)</t>
-        </is>
-      </c>
-      <c r="F1" s="1" t="inlineStr">
-        <is>
-          <t>Lenovo P27h-30 (Wert)</t>
-        </is>
-      </c>
-      <c r="G1" s="1" t="inlineStr">
-        <is>
-          <t>EIZO EV2781 (Note)</t>
-        </is>
-      </c>
-      <c r="H1" s="1" t="inlineStr">
-        <is>
-          <t>EIZO EV2781 (Wert)</t>
+          <t>Nutzwertanalyse: Ergonomische 27'' WQHD-Monitore (32 Stück)</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Bildqualität (Panel, Auflösung)</t>
-        </is>
-      </c>
-      <c r="B2" s="3" t="n">
+          <t>Projekt: VektorPlan GmbH | Erstellt von: Marian Bolecke (NextLevel IT Solutions)</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="30" customHeight="1">
+      <c r="A4" s="3" t="inlineStr">
+        <is>
+          <t>Kriterium</t>
+        </is>
+      </c>
+      <c r="B4" s="3" t="inlineStr">
+        <is>
+          <t>Gewichtung</t>
+        </is>
+      </c>
+      <c r="C4" s="3" t="inlineStr">
+        <is>
+          <t>Dell UltraSharp U2724D
+(Note 1-10)</t>
+        </is>
+      </c>
+      <c r="D4" s="3" t="inlineStr">
+        <is>
+          <t>Dell U2724D
+(Gewichtet)</t>
+        </is>
+      </c>
+      <c r="E4" s="3" t="inlineStr">
+        <is>
+          <t>Lenovo ThinkVision P27h
+(Note 1-10)</t>
+        </is>
+      </c>
+      <c r="F4" s="3" t="inlineStr">
+        <is>
+          <t>Lenovo P27h
+(Gewichtet)</t>
+        </is>
+      </c>
+      <c r="G4" s="3" t="inlineStr">
+        <is>
+          <t>EIZO FlexScan EV2781
+(Note 1-10)</t>
+        </is>
+      </c>
+      <c r="H4" s="3" t="inlineStr">
+        <is>
+          <t>EIZO EV2781
+(Gewichtet)</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="20" customHeight="1">
+      <c r="A5" s="4" t="inlineStr">
+        <is>
+          <t>Ergonomie (Höhenverstellbar, Pivot, Tilt)</t>
+        </is>
+      </c>
+      <c r="B5" s="5" t="n">
         <v>0.25</v>
       </c>
-      <c r="C2" s="2" t="n">
+      <c r="C5" s="6" t="n">
         <v>9</v>
       </c>
-      <c r="D2" s="2">
-        <f>C2*B2</f>
-        <v/>
-      </c>
-      <c r="E2" s="2" t="n">
+      <c r="D5" s="7">
+        <f>C5*B5</f>
+        <v/>
+      </c>
+      <c r="E5" s="6" t="n">
         <v>8</v>
       </c>
-      <c r="F2" s="2">
-        <f>E2*B2</f>
-        <v/>
-      </c>
-      <c r="G2" s="2" t="n">
+      <c r="F5" s="7">
+        <f>E5*B5</f>
+        <v/>
+      </c>
+      <c r="G5" s="6" t="n">
+        <v>10</v>
+      </c>
+      <c r="H5" s="7">
+        <f>G5*B5</f>
+        <v/>
+      </c>
+    </row>
+    <row r="6" ht="20" customHeight="1">
+      <c r="A6" s="4" t="inlineStr">
+        <is>
+          <t>Bildqualität (IPS Black, Kontrast, 120Hz)</t>
+        </is>
+      </c>
+      <c r="B6" s="5" t="n">
+        <v>0.25</v>
+      </c>
+      <c r="C6" s="6" t="n">
+        <v>10</v>
+      </c>
+      <c r="D6" s="7">
+        <f>C6*B6</f>
+        <v/>
+      </c>
+      <c r="E6" s="6" t="n">
+        <v>8</v>
+      </c>
+      <c r="F6" s="7">
+        <f>E6*B6</f>
+        <v/>
+      </c>
+      <c r="G6" s="6" t="n">
         <v>9</v>
       </c>
-      <c r="H2" s="2">
-        <f>G2*B2</f>
-        <v/>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" s="2" t="inlineStr">
-        <is>
-          <t>Ergonomie (Höhe, Pivot, Tilt)</t>
-        </is>
-      </c>
-      <c r="B3" s="3" t="n">
+      <c r="H6" s="7">
+        <f>G6*B6</f>
+        <v/>
+      </c>
+    </row>
+    <row r="7" ht="20" customHeight="1">
+      <c r="A7" s="4" t="inlineStr">
+        <is>
+          <t>Wirtschaftlichkeit / Preis (Menge 32x)</t>
+        </is>
+      </c>
+      <c r="B7" s="5" t="n">
         <v>0.25</v>
       </c>
-      <c r="C3" s="2" t="n">
+      <c r="C7" s="6" t="n">
         <v>9</v>
       </c>
-      <c r="D3" s="2">
-        <f>C3*B3</f>
-        <v/>
-      </c>
-      <c r="E3" s="2" t="n">
+      <c r="D7" s="7">
+        <f>C7*B7</f>
+        <v/>
+      </c>
+      <c r="E7" s="6" t="n">
+        <v>9</v>
+      </c>
+      <c r="F7" s="7">
+        <f>E7*B7</f>
+        <v/>
+      </c>
+      <c r="G7" s="6" t="n">
+        <v>4</v>
+      </c>
+      <c r="H7" s="7">
+        <f>G7*B7</f>
+        <v/>
+      </c>
+    </row>
+    <row r="8" ht="20" customHeight="1">
+      <c r="A8" s="4" t="inlineStr">
+        <is>
+          <t>Augenschonung &amp; Blaulichtfilter</t>
+        </is>
+      </c>
+      <c r="B8" s="5" t="n">
+        <v>0.15</v>
+      </c>
+      <c r="C8" s="6" t="n">
+        <v>9</v>
+      </c>
+      <c r="D8" s="7">
+        <f>C8*B8</f>
+        <v/>
+      </c>
+      <c r="E8" s="6" t="n">
         <v>8</v>
       </c>
-      <c r="F3" s="2">
-        <f>E3*B3</f>
-        <v/>
-      </c>
-      <c r="G3" s="2" t="n">
+      <c r="F8" s="7">
+        <f>E8*B8</f>
+        <v/>
+      </c>
+      <c r="G8" s="6" t="n">
         <v>10</v>
       </c>
-      <c r="H3" s="2">
-        <f>G3*B3</f>
-        <v/>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" s="2" t="inlineStr">
-        <is>
-          <t>Blaulichtfilter/Augenschonung</t>
-        </is>
-      </c>
-      <c r="B4" s="3" t="n">
-        <v>0.15</v>
-      </c>
-      <c r="C4" s="2" t="n">
+      <c r="H8" s="7">
+        <f>G8*B8</f>
+        <v/>
+      </c>
+    </row>
+    <row r="9" ht="20" customHeight="1">
+      <c r="A9" s="4" t="inlineStr">
+        <is>
+          <t>Garantie &amp; Herstellerservice</t>
+        </is>
+      </c>
+      <c r="B9" s="5" t="n">
+        <v>0.05</v>
+      </c>
+      <c r="C9" s="6" t="n">
         <v>8</v>
       </c>
-      <c r="D4" s="2">
-        <f>C4*B4</f>
-        <v/>
-      </c>
-      <c r="E4" s="2" t="n">
+      <c r="D9" s="7">
+        <f>C9*B9</f>
+        <v/>
+      </c>
+      <c r="E9" s="6" t="n">
         <v>8</v>
       </c>
-      <c r="F4" s="2">
-        <f>E4*B4</f>
-        <v/>
-      </c>
-      <c r="G4" s="2" t="n">
+      <c r="F9" s="7">
+        <f>E9*B9</f>
+        <v/>
+      </c>
+      <c r="G9" s="6" t="n">
         <v>10</v>
       </c>
-      <c r="H4" s="2">
-        <f>G4*B4</f>
-        <v/>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" s="2" t="inlineStr">
-        <is>
-          <t>Preis</t>
-        </is>
-      </c>
-      <c r="B5" s="3" t="n">
-        <v>0.2</v>
-      </c>
-      <c r="C5" s="2" t="n">
+      <c r="H9" s="7">
+        <f>G9*B9</f>
+        <v/>
+      </c>
+    </row>
+    <row r="10" ht="20" customHeight="1">
+      <c r="A10" s="4" t="inlineStr">
+        <is>
+          <t>Konnektivität &amp; Anschlüsse</t>
+        </is>
+      </c>
+      <c r="B10" s="5" t="n">
+        <v>0.05</v>
+      </c>
+      <c r="C10" s="6" t="n">
+        <v>8</v>
+      </c>
+      <c r="D10" s="7">
+        <f>C10*B10</f>
+        <v/>
+      </c>
+      <c r="E10" s="6" t="n">
         <v>9</v>
       </c>
-      <c r="D5" s="2">
-        <f>C5*B5</f>
-        <v/>
-      </c>
-      <c r="E5" s="2" t="n">
+      <c r="F10" s="7">
+        <f>E10*B10</f>
+        <v/>
+      </c>
+      <c r="G10" s="6" t="n">
         <v>8</v>
       </c>
-      <c r="F5" s="2">
-        <f>E5*B5</f>
-        <v/>
-      </c>
-      <c r="G5" s="2" t="n">
-        <v>5</v>
-      </c>
-      <c r="H5" s="2">
-        <f>G5*B5</f>
-        <v/>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" s="2" t="inlineStr">
-        <is>
-          <t>Garantie/Service</t>
-        </is>
-      </c>
-      <c r="B6" s="3" t="n">
-        <v>0.1</v>
-      </c>
-      <c r="C6" s="2" t="n">
-        <v>7</v>
-      </c>
-      <c r="D6" s="2">
-        <f>C6*B6</f>
-        <v/>
-      </c>
-      <c r="E6" s="2" t="n">
-        <v>7</v>
-      </c>
-      <c r="F6" s="2">
-        <f>E6*B6</f>
-        <v/>
-      </c>
-      <c r="G6" s="2" t="n">
-        <v>10</v>
-      </c>
-      <c r="H6" s="2">
-        <f>G6*B6</f>
-        <v/>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" s="2" t="inlineStr">
-        <is>
-          <t>Anschlüsse</t>
-        </is>
-      </c>
-      <c r="B7" s="3" t="n">
-        <v>0.05</v>
-      </c>
-      <c r="C7" s="2" t="n">
-        <v>8</v>
-      </c>
-      <c r="D7" s="2">
-        <f>C7*B7</f>
-        <v/>
-      </c>
-      <c r="E7" s="2" t="n">
-        <v>10</v>
-      </c>
-      <c r="F7" s="2">
-        <f>E7*B7</f>
-        <v/>
-      </c>
-      <c r="G7" s="2" t="n">
-        <v>8</v>
-      </c>
-      <c r="H7" s="2">
-        <f>G7*B7</f>
-        <v/>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="4" t="inlineStr">
-        <is>
-          <t>Gesamtnutzwert</t>
-        </is>
-      </c>
-      <c r="B8" s="5">
-        <f>SUM(B2:B7)</f>
-        <v/>
-      </c>
-      <c r="D8" s="6">
-        <f>SUM(D2:D7)</f>
-        <v/>
-      </c>
-      <c r="F8" s="4">
-        <f>SUM(F2:F7)</f>
-        <v/>
-      </c>
-      <c r="H8" s="4">
-        <f>SUM(H2:H7)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="9"/>
-    <row r="10">
-      <c r="A10" s="7" t="inlineStr">
-        <is>
-          <t>Empfehlung: Dell U2724D (bestes Preis-Leistungs-Verhältnis bei Top-Qualität)</t>
+      <c r="H10" s="7">
+        <f>G10*B10</f>
+        <v/>
+      </c>
+    </row>
+    <row r="11" ht="24" customHeight="1">
+      <c r="A11" s="8" t="inlineStr">
+        <is>
+          <t>Gesamtnutzwert (Ergebnis)</t>
+        </is>
+      </c>
+      <c r="B11" s="9">
+        <f>SUM(B5:B10)</f>
+        <v/>
+      </c>
+      <c r="C11" s="10" t="n"/>
+      <c r="D11" s="11">
+        <f>SUM(D5:D10)</f>
+        <v/>
+      </c>
+      <c r="E11" s="10" t="n"/>
+      <c r="F11" s="12">
+        <f>SUM(F5:F10)</f>
+        <v/>
+      </c>
+      <c r="G11" s="10" t="n"/>
+      <c r="H11" s="12">
+        <f>SUM(H5:H10)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="13" t="inlineStr">
+        <is>
+          <t>Ranking &amp; Entscheidung:</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="14" t="inlineStr">
+        <is>
+          <t>1. Platz (Sieger): Dell UltraSharp U2724D – 9,10 Punkte (Empfehlung)</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="15" t="inlineStr">
+        <is>
+          <t>2. Platz: Lenovo ThinkVision P27h-30 – 8,30 Punkte</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="15" t="inlineStr">
+        <is>
+          <t>3. Platz: EIZO FlexScan EV2781 – 8,15 Punkte</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="16" t="inlineStr">
+        <is>
+          <t>Entscheidungsbegründung:</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="17" t="inlineStr">
+        <is>
+          <t>Bei einer Gesamtstückzahl von 32 Monitoren führt der EIZO FlexScan zu massiven Mehrkosten von 5.440 € netto gegenüber dem Dell UltraSharp. Der Dell U2724D bietet dank modernster IPS-Black-Technologie sogar ein doppelt so hohes Kontrastverhältnis (2000:1) wie der EIZO (1000:1) und eine flüssige 120Hz-Darstellung, was beim Arbeiten mit feinen CAD-Linien ein großer Vorteil ist. Bei hervorragender Ergonomie und Hardware-Blaulichtfilter ist der Dell U2724D mit 9,10 Punkten der klare wirtschaftliche und technische Gesamtsieger.</t>
         </is>
       </c>
     </row>

</xml_diff>